<commit_message>
Code Updation For Emulator Comapatibility
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Modules/01_Login/CompanyLogin/01_CompanyLoginTest.xlsx
+++ b/src/test/resources/testdata/Modules/01_Login/CompanyLogin/01_CompanyLoginTest.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\testing\Documents\Bandhan_World_APPIUM\src\test\resources\testdata\Modules\01_Login\CompanyLogin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EADD90E-5EEF-4DB4-8BDD-8CAE86D91395}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B819941-7541-4D78-9681-5BDAE21A6AF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{D5674106-8292-4F40-9DFC-E6EAC771FC2F}"/>
   </bookViews>
@@ -90,19 +90,20 @@
 verifycompanyerrormessage</t>
   </si>
   <si>
+    <t>bandhaninftest</t>
+  </si>
+  <si>
+    <t>01_CompanyLogin</t>
+  </si>
+  <si>
+    <t>2602000005</t>
+  </si>
+  <si>
     <t>entercompanyname
 clicksubmitbutton
 hidekeyboard
+relaunchapp
 verifychooselanguagepagedisplay</t>
-  </si>
-  <si>
-    <t>bandhaninftest</t>
-  </si>
-  <si>
-    <t>01_CompanyLogin</t>
-  </si>
-  <si>
-    <t>2602000005</t>
   </si>
 </sst>
 </file>
@@ -1076,10 +1077,10 @@
     </row>
     <row r="2" spans="1:8" ht="87" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>6</v>
@@ -1100,10 +1101,10 @@
     </row>
     <row r="3" spans="1:8" ht="58" x14ac:dyDescent="0.35">
       <c r="A3" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>7</v>
@@ -1124,12 +1125,12 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="58" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A4" s="8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>8</v>
@@ -1138,10 +1139,10 @@
         <v>9</v>
       </c>
       <c r="E4" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F4" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>10</v>

</xml_diff>